<commit_message>
Update playwright config and add new API test cases
</commit_message>
<xml_diff>
--- a/tests/TestData/OrangeHRM_Login_All_Test.xlsx
+++ b/tests/TestData/OrangeHRM_Login_All_Test.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Training_Scripts\Playwright_Training_NewVersion\tests\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93AA6A3D-AE2E-459B-8DF2-CF6625201EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910EB4DA-D74B-4E06-81DC-BBA35A091186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{26C72732-9E7C-472C-B662-0D62840774E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>test_case</t>
   </si>
@@ -70,6 +72,9 @@
   </si>
   <si>
     <t>Required</t>
+  </si>
+  <si>
+    <t>admin1234</t>
   </si>
 </sst>
 </file>
@@ -496,7 +501,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>13</v>
@@ -529,4 +534,22 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAE7753B-0150-48AE-B0B5-5071B2FD3A75}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D78509F3-9C87-4297-9C5F-F9A0CAD25D88}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>